<commit_message>
saving minor edits to o&m costs spreadsheet
</commit_message>
<xml_diff>
--- a/data/om_costs/IPTDS O&M Costs 20240409.xlsx
+++ b/data/om_costs/IPTDS O&M Costs 20240409.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Git\SnakeRiverIPTDS\data\om_costs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{283320DD-1E00-4BA7-91FC-84ED55454DAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41A97F15-27C3-4059-86F2-A9AEB9BA3380}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -488,7 +488,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2136" uniqueCount="443">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2137" uniqueCount="444">
   <si>
     <t>WDFW</t>
   </si>
@@ -1855,6 +1855,9 @@
   </si>
   <si>
     <t>SW1, SW2, LAP, WR2, MR1, WEN, ACM</t>
+  </si>
+  <si>
+    <t>Completed</t>
   </si>
 </sst>
 </file>
@@ -2146,7 +2149,7 @@
     <xf numFmtId="44" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="147">
+  <cellXfs count="149">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -2499,6 +2502,12 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -2989,7 +2998,9 @@
       <c r="H2" s="118" t="s">
         <v>378</v>
       </c>
-      <c r="J2" s="136"/>
+      <c r="J2" s="148" t="s">
+        <v>443</v>
+      </c>
       <c r="K2" s="136"/>
       <c r="L2" s="136"/>
       <c r="M2" s="136"/>
@@ -3204,7 +3215,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="J5" s="106" t="s">
+      <c r="J5" s="147" t="s">
         <v>237</v>
       </c>
       <c r="K5" s="106" t="s">
@@ -3536,7 +3547,7 @@
         <f t="shared" si="0"/>
         <v>15225.039999999999</v>
       </c>
-      <c r="J9" s="106" t="s">
+      <c r="J9" s="147" t="s">
         <v>86</v>
       </c>
       <c r="K9" s="106" t="s">
@@ -4710,7 +4721,7 @@
       </c>
     </row>
     <row r="28" spans="4:28" ht="20.399999999999999" x14ac:dyDescent="0.3">
-      <c r="J28" s="106" t="s">
+      <c r="J28" s="147" t="s">
         <v>90</v>
       </c>
       <c r="K28" s="112" t="s">
@@ -4769,7 +4780,7 @@
       </c>
     </row>
     <row r="29" spans="4:28" x14ac:dyDescent="0.3">
-      <c r="J29" s="106" t="s">
+      <c r="J29" s="147" t="s">
         <v>83</v>
       </c>
       <c r="K29" s="112" t="s">

</xml_diff>